<commit_message>
Add February ITNOW Nowcast
</commit_message>
<xml_diff>
--- a/static/ITNOW/ITNOW_History.xlsx
+++ b/static/ITNOW/ITNOW_History.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreaviselli/Documents/GitHub/andreaviselli.github.io/static/ITNOW/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4C432B4-A52F-264F-978D-F81F53A3B9B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DFFA4F3-C334-B64C-BE1C-D5C22CE806BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3700" yWindow="-21100" windowWidth="38400" windowHeight="21100" xr2:uid="{6515F016-35AB-974D-935F-759783D4EEB3}"/>
+    <workbookView xWindow="0" yWindow="9020" windowWidth="29400" windowHeight="10100" activeTab="1" xr2:uid="{6515F016-35AB-974D-935F-759783D4EEB3}"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="96">
   <si>
     <t>Nowcast</t>
   </si>
@@ -770,12 +770,6 @@
     <xf numFmtId="0" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -846,6 +840,15 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -876,14 +879,11 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1245,88 +1245,88 @@
       </c>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="40" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="16"/>
+      <c r="B3" s="41"/>
     </row>
     <row r="4" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="18" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="18" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="18" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="18" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="18" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="18" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="18" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="18" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="16" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1446,10 +1446,36 @@
       </c>
     </row>
     <row r="4" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
+      <c r="A4" s="5">
+        <v>46099</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="6">
+        <v>2</v>
+      </c>
+      <c r="D4" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E4" s="4">
+        <v>1.4E-3</v>
+      </c>
+      <c r="F4" s="4">
+        <v>1.6999999999999999E-3</v>
+      </c>
+      <c r="G4" s="4">
+        <v>-4.1999999999999997E-3</v>
+      </c>
+      <c r="H4" s="4">
+        <v>9.4000000000000004E-3</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="5" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C5" s="8"/>
@@ -1476,407 +1502,407 @@
   <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.83203125" style="27" customWidth="1"/>
-    <col min="2" max="2" width="50.83203125" style="27" customWidth="1"/>
-    <col min="3" max="4" width="20.83203125" style="27" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" style="27" customWidth="1"/>
-    <col min="6" max="16384" width="10.83203125" style="27"/>
+    <col min="1" max="1" width="25.83203125" style="25" customWidth="1"/>
+    <col min="2" max="2" width="50.83203125" style="25" customWidth="1"/>
+    <col min="3" max="4" width="20.83203125" style="25" customWidth="1"/>
+    <col min="5" max="5" width="30.83203125" style="25" customWidth="1"/>
+    <col min="6" max="16384" width="10.83203125" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="39" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="53" t="s">
+      <c r="B1" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
     </row>
     <row r="2" spans="1:5" ht="19" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="D2" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="26" t="s">
+      <c r="E2" s="24" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="30" t="s">
+      <c r="C3" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="D3" s="30">
+      <c r="D3" s="28">
         <v>2</v>
       </c>
-      <c r="E3" s="31" t="s">
+      <c r="E3" s="29" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="31" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="C4" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="D4" s="34">
+      <c r="D4" s="32">
         <v>2</v>
       </c>
-      <c r="E4" s="35" t="s">
+      <c r="E4" s="33" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="34" t="s">
+      <c r="C5" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="34">
+      <c r="D5" s="32">
         <v>1</v>
       </c>
-      <c r="E5" s="35" t="s">
+      <c r="E5" s="33" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="D6" s="34">
+      <c r="D6" s="32">
         <v>1</v>
       </c>
-      <c r="E6" s="35" t="s">
+      <c r="E6" s="33" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="B7" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="C7" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="34">
+      <c r="D7" s="32">
         <v>2</v>
       </c>
-      <c r="E7" s="35" t="s">
+      <c r="E7" s="33" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="36" t="s">
+      <c r="B8" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="34">
+      <c r="D8" s="32">
         <v>1</v>
       </c>
-      <c r="E8" s="35" t="s">
+      <c r="E8" s="33" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="B9" s="36" t="s">
+      <c r="B9" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="D9" s="34">
+      <c r="D9" s="32">
         <v>1</v>
       </c>
-      <c r="E9" s="35" t="s">
+      <c r="E9" s="33" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A10" s="32" t="s">
+      <c r="A10" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="36" t="s">
+      <c r="B10" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="C10" s="34" t="s">
+      <c r="C10" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="D10" s="34">
+      <c r="D10" s="32">
         <v>0</v>
       </c>
-      <c r="E10" s="35" t="s">
+      <c r="E10" s="33" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="36" t="s">
+      <c r="B11" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="C11" s="34" t="s">
+      <c r="C11" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="D11" s="34">
+      <c r="D11" s="32">
         <v>0</v>
       </c>
-      <c r="E11" s="35" t="s">
+      <c r="E11" s="33" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A12" s="32" t="s">
+      <c r="A12" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="B12" s="36" t="s">
+      <c r="B12" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="C12" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="34">
+      <c r="D12" s="32">
         <v>2</v>
       </c>
-      <c r="E12" s="35" t="s">
+      <c r="E12" s="33" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="B13" s="36" t="s">
+      <c r="B13" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="C13" s="34" t="s">
+      <c r="C13" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="D13" s="34">
+      <c r="D13" s="32">
         <v>1</v>
       </c>
-      <c r="E13" s="35" t="s">
+      <c r="E13" s="33" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A14" s="32" t="s">
+      <c r="A14" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="B14" s="36" t="s">
+      <c r="B14" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="C14" s="34" t="s">
+      <c r="C14" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="34">
+      <c r="D14" s="32">
         <v>1</v>
       </c>
-      <c r="E14" s="35" t="s">
+      <c r="E14" s="33" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A15" s="32" t="s">
+      <c r="A15" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="B15" s="36" t="s">
+      <c r="B15" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="C15" s="34" t="s">
+      <c r="C15" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="D15" s="34">
+      <c r="D15" s="32">
         <v>2</v>
       </c>
-      <c r="E15" s="35" t="s">
+      <c r="E15" s="33" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A16" s="32" t="s">
+      <c r="A16" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="B16" s="36" t="s">
+      <c r="B16" s="34" t="s">
         <v>74</v>
       </c>
-      <c r="C16" s="34" t="s">
+      <c r="C16" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="D16" s="34">
+      <c r="D16" s="32">
         <v>1</v>
       </c>
-      <c r="E16" s="35" t="s">
+      <c r="E16" s="33" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A17" s="32" t="s">
+      <c r="A17" s="30" t="s">
         <v>76</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C17" s="34" t="s">
+      <c r="C17" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="D17" s="34">
+      <c r="D17" s="32">
         <v>0</v>
       </c>
-      <c r="E17" s="35" t="s">
+      <c r="E17" s="33" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A18" s="32" t="s">
+      <c r="A18" s="30" t="s">
         <v>78</v>
       </c>
-      <c r="B18" s="36" t="s">
+      <c r="B18" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="C18" s="34" t="s">
+      <c r="C18" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="D18" s="34">
+      <c r="D18" s="32">
         <v>0</v>
       </c>
-      <c r="E18" s="35" t="s">
+      <c r="E18" s="33" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A19" s="32" t="s">
+      <c r="A19" s="30" t="s">
         <v>81</v>
       </c>
-      <c r="B19" s="36" t="s">
+      <c r="B19" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="C19" s="34" t="s">
+      <c r="C19" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="D19" s="34">
+      <c r="D19" s="32">
         <v>0</v>
       </c>
-      <c r="E19" s="35" t="s">
+      <c r="E19" s="33" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A20" s="32" t="s">
+      <c r="A20" s="30" t="s">
         <v>83</v>
       </c>
-      <c r="B20" s="36" t="s">
+      <c r="B20" s="34" t="s">
         <v>84</v>
       </c>
-      <c r="C20" s="34" t="s">
+      <c r="C20" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="D20" s="34">
+      <c r="D20" s="32">
         <v>0</v>
       </c>
-      <c r="E20" s="35" t="s">
+      <c r="E20" s="33" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A21" s="32" t="s">
+      <c r="A21" s="30" t="s">
         <v>86</v>
       </c>
-      <c r="B21" s="36" t="s">
+      <c r="B21" s="34" t="s">
         <v>87</v>
       </c>
-      <c r="C21" s="34" t="s">
+      <c r="C21" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="D21" s="34">
+      <c r="D21" s="32">
         <v>0</v>
       </c>
-      <c r="E21" s="35" t="s">
+      <c r="E21" s="33" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A22" s="37" t="s">
+      <c r="A22" s="35" t="s">
         <v>88</v>
       </c>
-      <c r="B22" s="38" t="s">
+      <c r="B22" s="36" t="s">
         <v>89</v>
       </c>
-      <c r="C22" s="39" t="s">
+      <c r="C22" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="D22" s="39">
+      <c r="D22" s="37">
         <v>1</v>
       </c>
-      <c r="E22" s="40" t="s">
+      <c r="E22" s="38" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="41" t="s">
+      <c r="A23" s="42" t="s">
         <v>91</v>
       </c>
-      <c r="B23" s="42"/>
-      <c r="C23" s="42"/>
-      <c r="D23" s="42"/>
-      <c r="E23" s="43"/>
+      <c r="B23" s="43"/>
+      <c r="C23" s="43"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="44"/>
     </row>
     <row r="24" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="44" t="s">
+      <c r="A24" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="B24" s="45"/>
-      <c r="C24" s="45"/>
-      <c r="D24" s="46"/>
-      <c r="E24" s="47"/>
+      <c r="B24" s="46"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="47"/>
+      <c r="E24" s="48"/>
     </row>
     <row r="25" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="48" t="s">
+      <c r="A25" s="49" t="s">
         <v>93</v>
       </c>
-      <c r="B25" s="49"/>
-      <c r="C25" s="49"/>
-      <c r="D25" s="49"/>
-      <c r="E25" s="50"/>
+      <c r="B25" s="50"/>
+      <c r="C25" s="50"/>
+      <c r="D25" s="50"/>
+      <c r="E25" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Added forecast for Q1 and April
</commit_message>
<xml_diff>
--- a/static/ITNOW/ITNOW_History.xlsx
+++ b/static/ITNOW/ITNOW_History.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreaviselli/Documents/GitHub/andreaviselli.github.io/static/ITNOW/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DFFA4F3-C334-B64C-BE1C-D5C22CE806BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B58CDE46-2A1E-AD48-83D1-99CFFA6E8C21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="9020" windowWidth="29400" windowHeight="10100" activeTab="1" xr2:uid="{6515F016-35AB-974D-935F-759783D4EEB3}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="1" xr2:uid="{6515F016-35AB-974D-935F-759783D4EEB3}"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="97">
   <si>
     <t>Nowcast</t>
   </si>
@@ -405,12 +405,15 @@
     <t>Data information including the series acronym, exact and approximate publication delay expressed in months and weeks, and months, respectively, 
 and source used to generate nowcasts.</t>
   </si>
+  <si>
+    <t>Q1</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -523,6 +526,12 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Courier New"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
     </font>
   </fonts>
@@ -726,7 +735,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -884,6 +893,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="17" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1478,7 +1490,36 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C5" s="8"/>
+      <c r="A5" s="7">
+        <v>46125</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="C5" s="8">
+        <v>3</v>
+      </c>
+      <c r="D5" s="8">
+        <v>2026</v>
+      </c>
+      <c r="E5" s="4">
+        <v>1.5E-3</v>
+      </c>
+      <c r="F5" s="4">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G5" s="4">
+        <v>-5.7000000000000002E-3</v>
+      </c>
+      <c r="H5" s="4">
+        <v>8.8999999999999999E-3</v>
+      </c>
+      <c r="I5" s="4">
+        <v>5.4999999999999997E-3</v>
+      </c>
+      <c r="J5" s="54" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="6" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C6" s="8"/>

</xml_diff>

<commit_message>
Add ITNOW April Update
</commit_message>
<xml_diff>
--- a/static/ITNOW/ITNOW_History.xlsx
+++ b/static/ITNOW/ITNOW_History.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreaviselli/Documents/GitHub/andreaviselli.github.io/static/ITNOW/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B58CDE46-2A1E-AD48-83D1-99CFFA6E8C21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{345B9D0F-E5CA-0B4A-B7C4-4E176786F8FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="1" xr2:uid="{6515F016-35AB-974D-935F-759783D4EEB3}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="97">
   <si>
     <t>Nowcast</t>
   </si>
@@ -852,6 +852,9 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="10" fontId="17" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -893,9 +896,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="17" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1257,10 +1257,10 @@
       </c>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="41" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="41"/>
+      <c r="B3" s="42"/>
     </row>
     <row r="4" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="17" t="s">
@@ -1517,12 +1517,41 @@
       <c r="I5" s="4">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="J5" s="54" t="s">
+      <c r="J5" s="40" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C6" s="8"/>
+      <c r="A6" s="7">
+        <v>46151</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="8">
+        <v>4</v>
+      </c>
+      <c r="D6" s="8">
+        <v>2026</v>
+      </c>
+      <c r="E6" s="4">
+        <v>1.8E-3</v>
+      </c>
+      <c r="F6" s="4">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="G6" s="4">
+        <v>-6.4000000000000003E-3</v>
+      </c>
+      <c r="H6" s="4">
+        <v>1.06E-2</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="J6" s="4">
+        <v>1.0447E-3</v>
+      </c>
     </row>
     <row r="7" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C7" s="8"/>
@@ -1554,12 +1583,12 @@
       <c r="A1" s="39" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="52" t="s">
+      <c r="B1" s="53" t="s">
         <v>95</v>
       </c>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
     </row>
     <row r="2" spans="1:5" ht="19" x14ac:dyDescent="0.2">
       <c r="A2" s="20" t="s">
@@ -1919,31 +1948,31 @@
       </c>
     </row>
     <row r="23" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="42" t="s">
+      <c r="A23" s="43" t="s">
         <v>91</v>
       </c>
-      <c r="B23" s="43"/>
-      <c r="C23" s="43"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="44"/>
+      <c r="B23" s="44"/>
+      <c r="C23" s="44"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="45"/>
     </row>
     <row r="24" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="45" t="s">
+      <c r="A24" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="B24" s="46"/>
-      <c r="C24" s="46"/>
-      <c r="D24" s="47"/>
-      <c r="E24" s="48"/>
+      <c r="B24" s="47"/>
+      <c r="C24" s="47"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="49"/>
     </row>
     <row r="25" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="49" t="s">
+      <c r="A25" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="B25" s="50"/>
-      <c r="C25" s="50"/>
-      <c r="D25" s="50"/>
-      <c r="E25" s="51"/>
+      <c r="B25" s="51"/>
+      <c r="C25" s="51"/>
+      <c r="D25" s="51"/>
+      <c r="E25" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1954,4 +1983,10 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{9641a79b-5684-4ff8-89b0-3b715ae642f9}" enabled="1" method="Privileged" siteId="{adee44b2-91fc-40f1-abdd-9cc29351b5fd}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Update ITNOW page to full BG nowcast
</commit_message>
<xml_diff>
--- a/static/ITNOW/ITNOW_History.xlsx
+++ b/static/ITNOW/ITNOW_History.xlsx
@@ -1406,16 +1406,16 @@
         <v>2026</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0023</v>
+        <v>0.0013</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0053</v>
+        <v>0.0042</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0015</v>
+        <v>-0.0069</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0133</v>
+        <v>0.0176</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
ITNOW June 2026 Update
</commit_message>
<xml_diff>
--- a/static/ITNOW/ITNOW_History.xlsx
+++ b/static/ITNOW/ITNOW_History.xlsx
@@ -1429,7 +1429,42 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="C8" s="8" t="n"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.004500000000000001</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.0042</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-0.006999999999999999</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.0169</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.0122</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="C9" s="8" t="n"/>

</xml_diff>